<commit_message>
feat: add pure LSTM branch and integrate into train/evaluate scripts
</commit_message>
<xml_diff>
--- a/results/网络拟合情况.xlsx
+++ b/results/网络拟合情况.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\神经网络训练\underwater_robot_control\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C9E229A-49C4-4805-93BA-5E8CBB244F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF6CD44-C0A8-40BE-A4BB-3D81D03D4D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="40">
   <si>
     <r>
       <rPr>
@@ -280,25 +280,57 @@
     <t>理论公式计算</t>
   </si>
   <si>
-    <t>[6.159,2.272,15.263,5.468,3.493,12.923]</t>
-  </si>
-  <si>
-    <t>[5.078,1.736,10.181,3.958,2.555,9.878]</t>
-  </si>
-  <si>
-    <t>[0.0827 0.0557 0.0579 0.5055 1.0066 1.7802]</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>[0.0515 0.0391 0.0401 0.2794 0.4272 0.78  ]</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>[0.149, 0.161, 0.115, 1.23, 1.19, 2.544]</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>[0.104, 0.114, 0.080, 0.289, 0.279, 0.480]</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>[0.0967 0.0937 0.0989 0.8319 0.8997 1.1998]</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>[0.0663 0.0617 0.0697 0.4029 0.4391 0.5529]</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>[6.159,2.272,15.263,319.604,196.568,229.957]</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>[5.078,1.736,10.181,231.985,141.130,153.825]</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>纯</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>LSTM</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>[0.0381 0.0599 0.0955 0.1129 0.1343 0.1119]</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>[0.0298 0.0534 0.0669 0.0835 0.0973 0.1006]</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -306,7 +338,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -332,6 +364,13 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -649,6 +688,7 @@
     <col min="5" max="6" width="36.625" customWidth="1"/>
     <col min="7" max="7" width="37.125" customWidth="1"/>
     <col min="8" max="9" width="36.625" customWidth="1"/>
+    <col min="10" max="10" width="21.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.15">
@@ -809,7 +849,7 @@
         <v>17</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>18</v>
@@ -836,7 +876,7 @@
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>24</v>
@@ -883,7 +923,7 @@
         <v>0.21487742662429801</v>
       </c>
       <c r="I10" s="1">
-        <v>0.86132311820983798</v>
+        <v>0.70343935489654497</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15" x14ac:dyDescent="0.15">
@@ -895,9 +935,15 @@
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:9" ht="15" x14ac:dyDescent="0.15">
       <c r="C14" s="4" t="s">
         <v>30</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.15">
@@ -908,32 +954,56 @@
       <c r="C15" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="D15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="15" x14ac:dyDescent="0.15">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+        <v>35</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.15">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="15" x14ac:dyDescent="0.15">
+        <v>36</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.15">
       <c r="A18" s="1" t="s">
         <v>29</v>
+      </c>
+      <c r="D18" s="1">
+        <v>9.7869540000000005E-2</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.70343935489654497</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>